<commit_message>
Ajustada a lógica de importação do Efetivo via Excel para capturar e salvar corretamente a coluna "Nº de Ordem"
</commit_message>
<xml_diff>
--- a/utilitarios-dev/efetivo.xlsx
+++ b/utilitarios-dev/efetivo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alan Kleber\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\projetos\GSVR\utilitarios-dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B191A72A-664F-4521-AB4E-15CF34F71A69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D843BDA7-3608-40A9-B4B3-09E03359BF3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5F3109F1-C52A-4153-9483-D0AAB607A092}"/>
   </bookViews>
@@ -6773,7 +6773,8 @@
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="22" max="24" width="9.28515625" bestFit="1" customWidth="1"/>

</xml_diff>